<commit_message>
Updated executablility and changed code to be in line with FB2503/CORE-002038. Retesting done
</commit_message>
<xml_diff>
--- a/rules/CORE-000790/negative/01/data/unit-test-coreid-FB2505-negative.xlsx
+++ b/rules/CORE-000790/negative/01/data/unit-test-coreid-FB2505-negative.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\verisian\core-contributor\rules\CORE-000790\negative\01\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\els_janssens\CORE\Rule_Authoring\core-contributor\rules\CORE-000790\negative\01\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2A98D1B-9956-4691-85CE-E7A58543DF3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3806A1A-C32F-47D2-AA15-EFC5A12B7272}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="1" r:id="rId1"/>
@@ -248,9 +248,6 @@
     <t>DM</t>
   </si>
   <si>
-    <t>015246-076-0003-00003</t>
-  </si>
-  <si>
     <t>076000300003</t>
   </si>
   <si>
@@ -296,9 +293,6 @@
     <t>BRA</t>
   </si>
   <si>
-    <t>015246-300-0004-00002</t>
-  </si>
-  <si>
     <t>300000400002</t>
   </si>
   <si>
@@ -329,9 +323,6 @@
     <t>GRC</t>
   </si>
   <si>
-    <t>015246-999-0004-9999</t>
-  </si>
-  <si>
     <t>99900049999</t>
   </si>
   <si>
@@ -341,9 +332,6 @@
     <t>Y</t>
   </si>
   <si>
-    <t>ZZZ100</t>
-  </si>
-  <si>
     <t>88800088888</t>
   </si>
   <si>
@@ -498,6 +486,18 @@
   </si>
   <si>
     <t>Record</t>
+  </si>
+  <si>
+    <t>123</t>
+  </si>
+  <si>
+    <t>124</t>
+  </si>
+  <si>
+    <t>125</t>
+  </si>
+  <si>
+    <t>126</t>
   </si>
 </sst>
 </file>
@@ -506,7 +506,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0;[Red]0"/>
-    <numFmt numFmtId="166" formatCode="yyyy\-mm\-dd;@"/>
+    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -610,7 +610,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -654,10 +654,7 @@
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1051,7 +1048,7 @@
         <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="D2">
         <v>5</v>
@@ -1060,7 +1057,7 @@
         <v>37</v>
       </c>
       <c r="F2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -1071,7 +1068,7 @@
         <v>6</v>
       </c>
       <c r="C3" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="D3">
         <v>5</v>
@@ -1080,7 +1077,7 @@
         <v>39</v>
       </c>
       <c r="F3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -1091,7 +1088,7 @@
         <v>6</v>
       </c>
       <c r="C4" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="D4">
         <v>6</v>
@@ -1100,7 +1097,7 @@
         <v>37</v>
       </c>
       <c r="F4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -1111,7 +1108,7 @@
         <v>6</v>
       </c>
       <c r="C5" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="D5">
         <v>6</v>
@@ -1120,7 +1117,7 @@
         <v>39</v>
       </c>
       <c r="F5" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -1131,7 +1128,7 @@
         <v>6</v>
       </c>
       <c r="C6" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="D6">
         <v>7</v>
@@ -1140,7 +1137,7 @@
         <v>37</v>
       </c>
       <c r="F6" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -1151,7 +1148,7 @@
         <v>6</v>
       </c>
       <c r="C7" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="D7">
         <v>7</v>
@@ -1160,7 +1157,7 @@
         <v>39</v>
       </c>
       <c r="F7" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
   </sheetData>
@@ -1172,6 +1169,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:AA8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="23" max="23" width="8.7109375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:27" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
@@ -1512,72 +1512,72 @@
       <c r="B5" t="s">
         <v>73</v>
       </c>
-      <c r="C5" s="18" t="s">
+      <c r="C5" s="8" t="s">
+        <v>154</v>
+      </c>
+      <c r="D5" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="E5" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="E5" s="8" t="s">
+      <c r="F5" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="F5" s="8" t="s">
+      <c r="G5" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="H5" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="I5" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="G5" s="8" t="s">
-        <v>76</v>
-      </c>
-      <c r="H5" s="8" t="s">
-        <v>77</v>
-      </c>
-      <c r="I5" s="8" t="s">
+      <c r="J5" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="J5" s="8" t="s">
-        <v>79</v>
-      </c>
       <c r="K5" s="9" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="L5" s="9"/>
       <c r="M5" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="N5" s="8" t="s">
         <v>80</v>
-      </c>
-      <c r="N5" s="8" t="s">
-        <v>81</v>
       </c>
       <c r="O5" s="10">
         <v>78</v>
       </c>
       <c r="P5" s="9"/>
       <c r="Q5" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="R5" s="8" t="s">
         <v>82</v>
       </c>
-      <c r="R5" s="8" t="s">
+      <c r="S5" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="S5" s="8" t="s">
+      <c r="T5" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="T5" s="8" t="s">
+      <c r="U5" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="U5" s="9" t="s">
+      <c r="V5" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="V5" s="7" t="s">
+      <c r="W5" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="W5" s="9" t="s">
-        <v>88</v>
-      </c>
       <c r="X5" s="7" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="Y5" s="9"/>
       <c r="Z5" s="8"/>
       <c r="AA5" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="6" spans="1:27" ht="60" x14ac:dyDescent="0.25">
@@ -1587,74 +1587,74 @@
       <c r="B6" t="s">
         <v>73</v>
       </c>
-      <c r="C6" s="18" t="s">
+      <c r="C6" s="8" t="s">
+        <v>155</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="E6" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="D6" s="8" t="s">
+      <c r="F6" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="E6" s="8" t="s">
+      <c r="G6" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="H6" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="I6" s="8" t="s">
         <v>92</v>
       </c>
-      <c r="F6" s="8" t="s">
+      <c r="J6" s="8" t="s">
         <v>93</v>
       </c>
-      <c r="G6" s="8" t="s">
-        <v>92</v>
-      </c>
-      <c r="H6" s="8" t="s">
+      <c r="K6" s="9" t="s">
         <v>93</v>
       </c>
-      <c r="I6" s="8" t="s">
+      <c r="L6" s="9" t="s">
         <v>94</v>
       </c>
-      <c r="J6" s="8" t="s">
+      <c r="M6" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="K6" s="9" t="s">
-        <v>95</v>
-      </c>
-      <c r="L6" s="9" t="s">
+      <c r="N6" s="8" t="s">
         <v>96</v>
-      </c>
-      <c r="M6" s="8" t="s">
-        <v>97</v>
-      </c>
-      <c r="N6" s="8" t="s">
-        <v>98</v>
       </c>
       <c r="O6" s="10">
         <v>70</v>
       </c>
       <c r="P6" s="9"/>
       <c r="Q6" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="R6" s="8" t="s">
         <v>82</v>
       </c>
-      <c r="R6" s="8" t="s">
+      <c r="S6" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="S6" s="8" t="s">
-        <v>84</v>
-      </c>
       <c r="T6" s="8" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="U6" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="V6" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="V6" s="7" t="s">
+      <c r="W6" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="W6" s="9" t="s">
-        <v>88</v>
-      </c>
       <c r="X6" s="7" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="Y6" s="9"/>
       <c r="Z6" s="8"/>
       <c r="AA6" s="8" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="7" spans="1:27" ht="60" x14ac:dyDescent="0.25">
@@ -1664,74 +1664,74 @@
       <c r="B7" t="s">
         <v>73</v>
       </c>
-      <c r="C7" s="18" t="s">
+      <c r="C7" s="8" t="s">
+        <v>156</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="G7" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="H7" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="I7" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="J7" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="K7" s="9" t="s">
+        <v>100</v>
+      </c>
+      <c r="L7" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="D7" s="8" t="s">
-        <v>102</v>
-      </c>
-      <c r="E7" s="8" t="s">
-        <v>92</v>
-      </c>
-      <c r="F7" s="8" t="s">
-        <v>93</v>
-      </c>
-      <c r="G7" s="8" t="s">
-        <v>92</v>
-      </c>
-      <c r="H7" s="8" t="s">
-        <v>93</v>
-      </c>
-      <c r="I7" s="8" t="s">
-        <v>94</v>
-      </c>
-      <c r="J7" s="8" t="s">
+      <c r="M7" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="K7" s="9" t="s">
-        <v>103</v>
-      </c>
-      <c r="L7" s="8" t="s">
-        <v>104</v>
-      </c>
-      <c r="M7" s="8" t="s">
-        <v>97</v>
-      </c>
       <c r="N7" s="8" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="O7" s="10">
         <v>71</v>
       </c>
       <c r="P7" s="9"/>
       <c r="Q7" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="R7" s="8" t="s">
         <v>82</v>
       </c>
-      <c r="R7" s="8" t="s">
+      <c r="S7" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="S7" s="8" t="s">
-        <v>84</v>
-      </c>
       <c r="T7" s="8" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="U7" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="V7" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="V7" s="7" t="s">
+      <c r="W7" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="W7" s="9" t="s">
-        <v>88</v>
-      </c>
       <c r="X7" s="7" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="Y7" s="9"/>
       <c r="Z7" s="8"/>
       <c r="AA7" s="8" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="8" spans="1:27" ht="60" x14ac:dyDescent="0.25">
@@ -1742,73 +1742,73 @@
         <v>73</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>105</v>
+        <v>157</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="E8" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="G8" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="H8" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="I8" s="8" t="s">
         <v>92</v>
       </c>
-      <c r="F8" s="8" t="s">
+      <c r="J8" s="8" t="s">
         <v>93</v>
       </c>
-      <c r="G8" s="8" t="s">
-        <v>92</v>
-      </c>
-      <c r="H8" s="8" t="s">
-        <v>93</v>
-      </c>
-      <c r="I8" s="8" t="s">
-        <v>94</v>
-      </c>
-      <c r="J8" s="8" t="s">
+      <c r="K8" s="9" t="s">
+        <v>100</v>
+      </c>
+      <c r="L8" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="M8" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="K8" s="9" t="s">
-        <v>103</v>
-      </c>
-      <c r="L8" s="8" t="s">
-        <v>104</v>
-      </c>
-      <c r="M8" s="8" t="s">
-        <v>97</v>
-      </c>
       <c r="N8" s="8" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="O8" s="10">
         <v>71</v>
       </c>
       <c r="P8" s="9"/>
       <c r="Q8" s="9" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="R8" s="8" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="S8" s="8" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="T8" s="8" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="U8" s="9" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="V8" s="9" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="W8" s="9" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="X8" s="9" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="Y8" s="9"/>
       <c r="Z8" s="8"/>
       <c r="AA8" s="8" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
     </row>
   </sheetData>
@@ -1820,6 +1820,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:R9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="15" max="16" width="16.140625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="11" t="s">
@@ -1832,49 +1835,49 @@
         <v>18</v>
       </c>
       <c r="D1" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="E1" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="F1" s="11" t="s">
+        <v>108</v>
+      </c>
+      <c r="G1" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="H1" s="11" t="s">
         <v>110</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="I1" s="11" t="s">
         <v>111</v>
       </c>
-      <c r="F1" s="11" t="s">
+      <c r="J1" s="11" t="s">
         <v>112</v>
       </c>
-      <c r="G1" s="11" t="s">
+      <c r="K1" s="11" t="s">
         <v>113</v>
       </c>
-      <c r="H1" s="11" t="s">
+      <c r="L1" s="11" t="s">
         <v>114</v>
       </c>
-      <c r="I1" s="11" t="s">
+      <c r="M1" s="12" t="s">
         <v>115</v>
       </c>
-      <c r="J1" s="11" t="s">
+      <c r="N1" s="12" t="s">
         <v>116</v>
       </c>
-      <c r="K1" s="11" t="s">
+      <c r="O1" s="11" t="s">
         <v>117</v>
       </c>
-      <c r="L1" s="11" t="s">
+      <c r="P1" s="11" t="s">
         <v>118</v>
       </c>
-      <c r="M1" s="12" t="s">
+      <c r="Q1" s="11" t="s">
         <v>119</v>
       </c>
-      <c r="N1" s="12" t="s">
+      <c r="R1" s="11" t="s">
         <v>120</v>
-      </c>
-      <c r="O1" s="11" t="s">
-        <v>121</v>
-      </c>
-      <c r="P1" s="11" t="s">
-        <v>122</v>
-      </c>
-      <c r="Q1" s="11" t="s">
-        <v>123</v>
-      </c>
-      <c r="R1" s="11" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="2" spans="1:18" ht="75" x14ac:dyDescent="0.25">
@@ -1888,49 +1891,49 @@
         <v>45</v>
       </c>
       <c r="D2" s="13" t="s">
+        <v>121</v>
+      </c>
+      <c r="E2" s="13" t="s">
+        <v>122</v>
+      </c>
+      <c r="F2" s="13" t="s">
+        <v>123</v>
+      </c>
+      <c r="G2" s="13" t="s">
+        <v>124</v>
+      </c>
+      <c r="H2" s="13" t="s">
         <v>125</v>
       </c>
-      <c r="E2" s="13" t="s">
+      <c r="I2" s="13" t="s">
         <v>126</v>
       </c>
-      <c r="F2" s="13" t="s">
+      <c r="J2" s="13" t="s">
         <v>127</v>
       </c>
-      <c r="G2" s="13" t="s">
+      <c r="K2" s="13" t="s">
         <v>128</v>
       </c>
-      <c r="H2" s="13" t="s">
+      <c r="L2" s="13" t="s">
         <v>129</v>
       </c>
-      <c r="I2" s="13" t="s">
+      <c r="M2" s="13" t="s">
+        <v>124</v>
+      </c>
+      <c r="N2" s="13" t="s">
+        <v>126</v>
+      </c>
+      <c r="O2" s="13" t="s">
         <v>130</v>
       </c>
-      <c r="J2" s="13" t="s">
+      <c r="P2" s="13" t="s">
         <v>131</v>
       </c>
-      <c r="K2" s="13" t="s">
+      <c r="Q2" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="L2" s="13" t="s">
+      <c r="R2" s="13" t="s">
         <v>133</v>
-      </c>
-      <c r="M2" s="13" t="s">
-        <v>128</v>
-      </c>
-      <c r="N2" s="13" t="s">
-        <v>130</v>
-      </c>
-      <c r="O2" s="13" t="s">
-        <v>134</v>
-      </c>
-      <c r="P2" s="13" t="s">
-        <v>135</v>
-      </c>
-      <c r="Q2" s="13" t="s">
-        <v>136</v>
-      </c>
-      <c r="R2" s="13" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.25">
@@ -2050,40 +2053,40 @@
         <v>72</v>
       </c>
       <c r="B5" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="D5">
         <v>1</v>
       </c>
       <c r="E5" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="F5" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="G5">
         <v>3</v>
       </c>
       <c r="I5" s="14" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="J5" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="K5" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="L5" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="M5" s="15">
         <v>0.1</v>
       </c>
       <c r="N5" s="16" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="O5" s="17">
         <v>40557</v>
@@ -2103,40 +2106,40 @@
         <v>72</v>
       </c>
       <c r="B6" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="D6">
         <v>1</v>
       </c>
       <c r="E6" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="F6" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="G6">
         <v>3</v>
       </c>
       <c r="I6" s="14" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="J6" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="K6" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="L6" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="M6" s="15">
         <v>0.1</v>
       </c>
       <c r="N6" s="16" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="O6" s="17">
         <v>40557</v>
@@ -2156,34 +2159,34 @@
         <v>72</v>
       </c>
       <c r="B7" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="D7">
         <v>1</v>
       </c>
       <c r="E7" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="F7" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="G7">
         <v>500</v>
       </c>
       <c r="I7" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="J7" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="K7" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="L7" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="O7" s="17">
         <v>40557</v>
@@ -2203,34 +2206,34 @@
         <v>72</v>
       </c>
       <c r="B8" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="D8">
         <v>2</v>
       </c>
       <c r="E8" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="F8" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="G8">
         <v>500</v>
       </c>
       <c r="I8" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="J8" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="K8" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="L8" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="O8" s="17">
         <v>40568</v>
@@ -2250,37 +2253,37 @@
         <v>72</v>
       </c>
       <c r="B9" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>105</v>
+        <v>157</v>
       </c>
       <c r="D9">
         <v>1</v>
       </c>
       <c r="F9" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="G9">
         <v>100</v>
       </c>
       <c r="I9" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="J9" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="K9" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="L9" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="O9" s="17" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="P9" s="17" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="Q9">
         <v>12</v>

</xml_diff>